<commit_message>
Added preparation_datetime to sample
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -1524,644 +1524,659 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>preparation_protocol</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>preparation_datetime</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>manufacturer</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>preparation_protocol</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>preparation_datetime</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>manufacturer</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>input_parameters</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>acquisition_datetime</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>input_data</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>microscope</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>experimenter</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>acquisition_protocol</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>data_reference</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>linked_references</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>field_illumination_images</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>microscope_collection</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>bit_depth</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>saturation_threshold</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>corner_fraction</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sigma</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>key_measurements</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>intensity_profiles</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>roi_profiles</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>roi_corners</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>roi_centers_of_mass</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>roi_centers_geometric</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>roi_centers_fitted</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>roi_centers_max_intensity</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>roi_center_region</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>processing_application</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>processing_version</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>processing_entity</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>processing_datetime</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>processing_log</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>warnings</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>errors</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>validation_datetime</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AY1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>image_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>image_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>channel_nr</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>channel_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>center_region_intensity_fraction</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>center_region_area_fraction</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>center_of_mass_y</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>center_of_mass_y_relative</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>center_of_mass_x</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>center_of_mass_x_relative</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>center_of_mass_distance_relative</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>center_geometric_y</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>center_geometric_y_relative</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>center_geometric_x</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>center_geometric_x_relative</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>center_geometric_distance_relative</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>center_fitted_y</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>center_fitted_y_relative</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>center_fitted_x</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>center_fitted_x_relative</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>center_fitted_distance_relative</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>max_intensity</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>max_intensity_pos_y</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>max_intensity_pos_y_relative</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>max_intensity_pos_x</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>max_intensity_pos_x_relative</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>max_intensity_distance_relative</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>top_left_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>top_left_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>top_center_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>top_center_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>top_right_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>top_right_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>middle_left_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>middle_left_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>middle_center_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>middle_center_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>middle_right_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>middle_right_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>bottom_left_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>bottom_left_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>bottom_center_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>bottom_center_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>bottom_right_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>bottom_right_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>table_data</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>data_reference</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>linked_references</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>bead_diameter_micron</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>preparation_protocol</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>preparation_datetime</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
         <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>preparation_protocol</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>manufacturer</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>sample</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>input_parameters</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>acquisition_datetime</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>input_data</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>output</t>
-        </is>
-      </c>
       <c r="F1" t="inlineStr">
-        <is>
-          <t>microscope</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>experimenter</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>acquisition_protocol</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>processed</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>data_reference</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>linked_references</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>field_illumination_images</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>microscope_collection</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>bit_depth</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>saturation_threshold</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>corner_fraction</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sigma</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet31.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:S1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>key_measurements</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>intensity_profiles</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>roi_profiles</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>roi_corners</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>roi_centers_of_mass</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>roi_centers_geometric</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>roi_centers_fitted</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>roi_centers_max_intensity</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>roi_center_region</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>comment</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>processing_application</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>processing_version</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>processing_entity</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>processing_datetime</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>processing_log</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>warnings</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>errors</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>validated</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>validation_datetime</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AY1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>image_name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>image_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>channel_name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>channel_nr</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>channel_id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>center_region_intensity_fraction</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>center_region_area_fraction</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>center_of_mass_y</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>center_of_mass_y_relative</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>center_of_mass_x</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>center_of_mass_x_relative</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>center_of_mass_distance_relative</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>center_geometric_y</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>center_geometric_y_relative</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>center_geometric_x</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>center_geometric_x_relative</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>center_geometric_distance_relative</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>center_fitted_y</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>center_fitted_y_relative</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>center_fitted_x</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>center_fitted_x_relative</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>center_fitted_distance_relative</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>max_intensity</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>max_intensity_pos_y</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>max_intensity_pos_y_relative</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>max_intensity_pos_x</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>max_intensity_pos_x_relative</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>max_intensity_distance_relative</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>top_left_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>top_left_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>top_center_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>top_center_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>top_right_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>top_right_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>middle_left_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>middle_left_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>middle_center_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>middle_center_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>middle_right_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>middle_right_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>bottom_left_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>bottom_left_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>bottom_center_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>bottom_center_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
-        <is>
-          <t>bottom_right_intensity_mean</t>
-        </is>
-      </c>
-      <c r="AT1" t="inlineStr">
-        <is>
-          <t>bottom_right_intensity_ratio</t>
-        </is>
-      </c>
-      <c r="AU1" t="inlineStr">
-        <is>
-          <t>table_data</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
-          <t>data_reference</t>
-        </is>
-      </c>
-      <c r="AW1" t="inlineStr">
-        <is>
-          <t>linked_references</t>
-        </is>
-      </c>
-      <c r="AX1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AY1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>bead_diameter_micron</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>preparation_protocol</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>manufacturer</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
@@ -3284,7 +3299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3295,15 +3310,20 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>preparation_datetime</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>manufacturer</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Renamed power_sample and associated terms to power_measurement
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -50,7 +50,7 @@
     <sheet name="LightSourcePowerInputParameters" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="LightSourcePowerOutput" sheetId="42" state="visible" r:id="rId42"/>
     <sheet name="LightSourcePowerKeyMeasurements" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="PowerSample" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet name="PowerMeasurement" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="LightSource" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="PowerMeter" sheetId="46" state="visible" r:id="rId46"/>
     <sheet name="LightSourcePower" sheetId="47" state="visible" r:id="rId47"/>
@@ -3016,7 +3016,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>power_samples</t>
+          <t>power_measurements</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>sampling_location</t>
+          <t>measuring_location</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">

</xml_diff>

<commit_message>
Renamed linearity to power_linearity Added short_term_power_stability and long_term_power_stability
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3115,7 +3115,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3151,30 +3151,40 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>linearity</t>
+          <t>power_linearity</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>short_term_power_stability</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>long_term_power_stability</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>table_data</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>data_reference</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>linked_references</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Added input_parameter short_long_term_threshold_seconds for power measurements to separate what short and long term stability means. Defaults to 1 sec Added output measurements for the duration of the measurements (short and long)
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3033,7 +3033,15 @@
   </sheetPr>
   <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>short_long_term_threshold_seconds</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3115,7 +3123,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3161,30 +3169,40 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>short_term_measurement_duration_seconds</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>long_term_power_stability</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>long_term_measurement_duration_seconds</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>table_data</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>data_reference</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>linked_references</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Moved measurement device to the power_measurement by ref
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3005,204 +3005,204 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>power_measurements</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>short_long_term_threshold_seconds</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>key_measurements</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>processing_application</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>processing_version</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>processing_entity</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>processing_datetime</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>processing_log</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>warnings</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>errors</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>validation_datetime</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>light_source</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>measurement_device</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>power_measurements</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet41.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>short_long_term_threshold_seconds</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet42.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>key_measurements</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>comment</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>processing_application</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>processing_version</t>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>power_mean_mw</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>power_median_mw</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>processing_entity</t>
+          <t>power_std_mw</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>processing_datetime</t>
+          <t>power_min_mw</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>processing_log</t>
+          <t>power_max_mw</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>warnings</t>
+          <t>power_linearity</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>errors</t>
+          <t>short_term_power_stability</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>validated</t>
+          <t>short_term_measurement_duration_seconds</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>validation_datetime</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet43.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>light_source</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>power_mean_mw</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>power_median_mw</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>power_std_mw</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>power_min_mw</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>power_max_mw</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>power_linearity</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>short_term_power_stability</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>short_term_measurement_duration_seconds</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
           <t>long_term_power_stability</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>long_term_measurement_duration_seconds</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>table_data</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>data_reference</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>linked_references</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Added the number of measurements for the light source power key measurements
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3118,7 +3118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:R1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3134,75 +3134,80 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>nr_of_measurements</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>power_mean_mw</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>power_median_mw</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>power_std_mw</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>power_min_mw</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>power_max_mw</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>power_linearity</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>short_term_power_stability</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>short_term_measurement_duration_seconds</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>long_term_power_stability</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>long_term_measurement_duration_seconds</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>table_data</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>data_reference</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>linked_references</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Added the measurement location for the light source power key measurements
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3118,7 +3118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R1"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3134,86 +3134,96 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>measuring_location</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>nr_of_measurements</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>power_mean_mw</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>power_median_mw</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>power_std_mw</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>power_min_mw</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>power_max_mw</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>power_linearity</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>short_term_power_stability</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>short_term_measurement_duration_seconds</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>long_term_power_stability</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>long_term_measurement_duration_seconds</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>table_data</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>data_reference</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>linked_references</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"SOURCE_EXIT,FIBER_EXIT,OBJECTIVE_BACKFOCAL,OBJECTIVE_EXIT,OBJECTIVE_FOCAL,OTHER"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Made LightSource a named_object Fixed some strategies to use composites strategies as arguments. Other minor corrections
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3290,13 +3290,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>wavelength_nm</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>description</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added more stats on linearity of power measurements
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3118,7 +3118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3169,50 +3169,70 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>power_linearity_slope</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>power_linearity_intercept</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>power_linearity_coefficient_of_determination</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>power_linearity_p_value</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>power_linearity_std_err</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
         <is>
           <t>short_term_power_stability</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>short_term_measurement_duration_seconds</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>long_term_power_stability</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>long_term_measurement_duration_seconds</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>table_data</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>data_reference</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>linked_references</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Modified light_source_power.yaml to detail input parameters defining stability measurements timing specs
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3026,13 +3026,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>short_long_term_threshold_seconds</t>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>short_term_stability_measurement_interval_seconds</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>short_term_stability_required_measurements</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>short_term_stability_required_integration_time_seconds</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>long_term_stability_measurement_interval_seconds</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>long_term_stability_required_measurements</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>long_term_stability_required_integration_time_seconds</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3179,40 +3204,30 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>short_term_measurement_duration_seconds</t>
+          <t>long_term_power_stability</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>long_term_power_stability</t>
+          <t>table_data</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>long_term_measurement_duration_seconds</t>
+          <t>data_reference</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>table_data</t>
+          <t>linked_references</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>data_reference</t>
+          <t>name</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
-        <is>
-          <t>linked_references</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Added the required number of measurements for linearity stats
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3026,36 +3026,41 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>linearity_required_measurements</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
         <is>
           <t>short_term_stability_measurement_interval_seconds</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>short_term_stability_required_measurements</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>short_term_stability_required_integration_time_seconds</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>long_term_stability_measurement_interval_seconds</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>long_term_stability_required_measurements</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>long_term_stability_required_integration_time_seconds</t>
         </is>

</xml_diff>

<commit_message>
Added the start and end datetimes of the linearity and stability measurements
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3148,7 +3148,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3199,60 +3199,90 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>power_linearity_start_datetime</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>power_linearity_end_datetime</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>power_linearity_slope</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>power_linearity_intercept</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>power_linearity_coefficient_of_determination</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>power_linearity_p_value</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>power_linearity_std_err</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>short_term_power_stability_start_datetime</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>short_term_power_stability_end_datetime</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
         <is>
           <t>short_term_power_stability</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>long_term_power_stability_start_datetime</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>long_term_power_stability_end_datetime</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
         <is>
           <t>long_term_power_stability</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>table_data</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>data_reference</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>linked_references</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>description</t>
         </is>

</xml_diff>

<commit_message>
Changed psf detection sigmas in xyz for sigma min and max for detection using LoG
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -2295,7 +2295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2316,30 +2316,25 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>sigma_z</t>
+          <t>sigma_min</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>sigma_y</t>
+          <t>sigma_max</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>sigma_x</t>
+          <t>snr_threshold</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>snr_threshold</t>
+          <t>fitting_r2_threshold</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
-        <is>
-          <t>fitting_r2_threshold</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
         <is>
           <t>intensity_robust_z_score_threshold</t>
         </is>

</xml_diff>

<commit_message>
Renamed measurement_device to power_meter
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3154,7 +3154,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>measurement_device</t>
+          <t>power_meter</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -3315,7 +3315,7 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>measurement_device</t>
+          <t>power_meter</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">

</xml_diff>

<commit_message>
Moved intensity_profiles to the core as used in multiple analysis instances
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -53,7 +53,13 @@
     <sheet name="PowerMeasurement" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="LightSource" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="PowerMeter" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="LightSourcePower" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="UserExperiment" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet name="UserExperimentDataset" sheetId="48" state="visible" r:id="rId48"/>
+    <sheet name="UserExperimentInputData" sheetId="49" state="visible" r:id="rId49"/>
+    <sheet name="UserExperimentInputParameters" sheetId="50" state="visible" r:id="rId50"/>
+    <sheet name="UserExperimentOutput" sheetId="51" state="visible" r:id="rId51"/>
+    <sheet name="UserExperimentKeyMeasurements" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="LightSourcePower" sheetId="53" state="visible" r:id="rId53"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1771,12 +1777,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>intensity_profiles</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>key_measurements</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>intensity_profiles</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -3457,6 +3463,118 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet48.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>input_parameters</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>acquisition_datetime</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>input_data</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>microscope</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>experimenter</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>acquisition_protocol</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>data_reference</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>linked_references</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet49.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>user_experiment_images</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>orthogonal_rois</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>profile_rois</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -3480,6 +3598,220 @@
       <c r="C1" t="inlineStr">
         <is>
           <t>url</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet50.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>bit_depth</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>saturation_threshold</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet51.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>intensity_profiles</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>orthogonal_images</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>fft_images</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>key_measurements</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>processing_application</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>processing_version</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>processing_entity</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>processing_datetime</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>processing_log</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>warnings</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>errors</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>validation_datetime</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet52.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>channel_nr</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>variation_coefficient</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>saturated_channels</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>table_data</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>data_reference</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>linked_references</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet53.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>preparation_protocol</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>preparation_datetime</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>manufacturer</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">

</xml_diff>

<commit_message>
Replacing key_measurements as a Table with a list of KeyMeasurement's. This provides: - More control on the slots - Ensures consistent nr of rows - Remover dataref and everything stays in the dataset file
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -38,18 +38,18 @@
     <sheet name="FieldIlluminationInputData" sheetId="29" state="visible" r:id="rId29"/>
     <sheet name="FieldIlluminationInputParameters" sheetId="30" state="visible" r:id="rId30"/>
     <sheet name="FieldIlluminationOutput" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="FieldIlluminationKeyMeasurements" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet name="FieldIlluminationKeyMeasurement" sheetId="32" state="visible" r:id="rId32"/>
     <sheet name="PSFBeads" sheetId="33" state="visible" r:id="rId33"/>
     <sheet name="PSFBeadsDataset" sheetId="34" state="visible" r:id="rId34"/>
     <sheet name="PSFBeadsInputData" sheetId="35" state="visible" r:id="rId35"/>
     <sheet name="PSFBeadsInputParameters" sheetId="36" state="visible" r:id="rId36"/>
     <sheet name="PSFBeadsOutput" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="PSFBeadsKeyMeasurements" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet name="PSFBeadsKeyMeasurement" sheetId="38" state="visible" r:id="rId38"/>
     <sheet name="LightSourcePowerDataset" sheetId="39" state="visible" r:id="rId39"/>
     <sheet name="LightSourcePowerInputData" sheetId="40" state="visible" r:id="rId40"/>
     <sheet name="LightSourcePowerInputParameters" sheetId="41" state="visible" r:id="rId41"/>
     <sheet name="LightSourcePowerOutput" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="LightSourcePowerKeyMeasurements" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet name="LightSourcePowerKeyMeasurement" sheetId="43" state="visible" r:id="rId43"/>
     <sheet name="PowerMeasurement" sheetId="44" state="visible" r:id="rId44"/>
     <sheet name="LightSource" sheetId="45" state="visible" r:id="rId45"/>
     <sheet name="PowerMeter" sheetId="46" state="visible" r:id="rId46"/>
@@ -58,7 +58,7 @@
     <sheet name="UserExperimentInputData" sheetId="49" state="visible" r:id="rId49"/>
     <sheet name="UserExperimentInputParameters" sheetId="50" state="visible" r:id="rId50"/>
     <sheet name="UserExperimentOutput" sheetId="51" state="visible" r:id="rId51"/>
-    <sheet name="UserExperimentKeyMeasurements" sheetId="52" state="visible" r:id="rId52"/>
+    <sheet name="UserExperimentKeyMeasurement" sheetId="52" state="visible" r:id="rId52"/>
     <sheet name="LightSourcePower" sheetId="53" state="visible" r:id="rId53"/>
   </sheets>
   <definedNames/>
@@ -1782,973 +1782,948 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>roi_profiles</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>roi_corners</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>roi_centers_of_mass</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>roi_centers_geometric</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>roi_centers_fitted</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>roi_centers_max_intensity</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>roi_center_region</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>key_measurements</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>roi_profiles</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>roi_corners</t>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>processing_application</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>processing_version</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>processing_entity</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>processing_datetime</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>processing_log</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>warnings</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>errors</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>validation_datetime</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AT1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>image_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>image_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>channel_nr</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>roi_centers_of_mass</t>
+          <t>channel_id</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>roi_centers_geometric</t>
+          <t>center_region_intensity_fraction</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>roi_centers_fitted</t>
+          <t>center_region_area_fraction</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>roi_centers_max_intensity</t>
+          <t>center_of_mass_y</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>roi_center_region</t>
+          <t>center_of_mass_y_relative</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>center_of_mass_x</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>center_of_mass_x_relative</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>center_of_mass_distance_relative</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>center_geometric_y</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>center_geometric_y_relative</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>center_geometric_x</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>center_geometric_x_relative</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>center_geometric_distance_relative</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>center_fitted_y</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>center_fitted_y_relative</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>center_fitted_x</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>center_fitted_x_relative</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>center_fitted_distance_relative</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>max_intensity</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>max_intensity_pos_y</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>max_intensity_pos_y_relative</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>max_intensity_pos_x</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>max_intensity_pos_x_relative</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>max_intensity_distance_relative</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>top_left_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>top_left_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>top_center_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>top_center_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>top_right_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>top_right_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>middle_left_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>middle_left_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>middle_center_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>middle_center_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>middle_right_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>middle_right_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>bottom_left_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>bottom_left_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>bottom_center_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>bottom_center_intensity_ratio</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>bottom_right_intensity_mean</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>bottom_right_intensity_ratio</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>bead_diameter_micron</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>preparation_protocol</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>preparation_datetime</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>manufacturer</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>sample</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>input_parameters</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>acquisition_datetime</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>input_data</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>output</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>microscope</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>experimenter</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>acquisition_protocol</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>processed</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>data_reference</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>linked_references</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>psf_beads_images</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>bit_depth</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>saturation_threshold</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>min_lateral_distance_factor</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>sigma_min</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>sigma_max</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>snr_threshold</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>fitting_r2_threshold</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>intensity_robust_z_score_threshold</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:X1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>analyzed_bead_centers</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_lateral_edge</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_self_proximity</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_axial_edge</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_intensity_outlier</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_z_fit_quality</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_y_fit_quality</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_x_fit_quality</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>bead_properties</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>bead_profiles_z</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>bead_profiles_y</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>bead_profiles_x</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>average_bead</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>key_measurements</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>comment</t>
         </is>
       </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>processing_application</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>processing_version</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>processing_entity</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>processing_datetime</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>processing_log</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>warnings</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>errors</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>validation_datetime</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:BO1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>channel_nr</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>total_bead_count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>considered_valid_count</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>considered_self_proximity_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>considered_lateral_edge_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>considered_axial_edge_count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>considered_intensity_outlier_count</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>considered_bad_fit_z_count</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>considered_bad_fit_y_count</t>
+        </is>
+      </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>processing_application</t>
+          <t>considered_bad_fit_x_count</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>processing_version</t>
+          <t>intensity_integrated_mean</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>processing_entity</t>
+          <t>intensity_integrated_median</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>processing_datetime</t>
+          <t>intensity_integrated_std</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>processing_log</t>
+          <t>intensity_max_mean</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>warnings</t>
+          <t>intensity_max_median</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>errors</t>
+          <t>intensity_max_std</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>validated</t>
+          <t>intensity_min_mean</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>validation_datetime</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet32.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:AY1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>image_name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>image_id</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>channel_name</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>channel_nr</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>channel_id</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>center_region_intensity_fraction</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>center_region_area_fraction</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>center_of_mass_y</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>center_of_mass_y_relative</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>center_of_mass_x</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>center_of_mass_x_relative</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>center_of_mass_distance_relative</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>center_geometric_y</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>center_geometric_y_relative</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>center_geometric_x</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>center_geometric_x_relative</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>center_geometric_distance_relative</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>center_fitted_y</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>center_fitted_y_relative</t>
+          <t>intensity_min_median</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>center_fitted_x</t>
+          <t>intensity_min_std</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>center_fitted_x_relative</t>
+          <t>intensity_std_mean</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>center_fitted_distance_relative</t>
+          <t>intensity_std_median</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>max_intensity</t>
+          <t>intensity_std_std</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>max_intensity_pos_y</t>
+          <t>fit_r2_z_mean</t>
         </is>
       </c>
       <c r="Y1" t="inlineStr">
         <is>
-          <t>max_intensity_pos_y_relative</t>
+          <t>fit_r2_z_median</t>
         </is>
       </c>
       <c r="Z1" t="inlineStr">
         <is>
-          <t>max_intensity_pos_x</t>
+          <t>fit_r2_z_std</t>
         </is>
       </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>max_intensity_pos_x_relative</t>
+          <t>fit_r2_y_mean</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>max_intensity_distance_relative</t>
+          <t>fit_r2_y_median</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>top_left_intensity_mean</t>
+          <t>fit_r2_y_std</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
         <is>
-          <t>top_left_intensity_ratio</t>
+          <t>fit_r2_x_mean</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>top_center_intensity_mean</t>
+          <t>fit_r2_x_median</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr">
         <is>
-          <t>top_center_intensity_ratio</t>
+          <t>fit_r2_x_std</t>
         </is>
       </c>
       <c r="AG1" t="inlineStr">
         <is>
-          <t>top_right_intensity_mean</t>
+          <t>fwhm_pixel_z_mean</t>
         </is>
       </c>
       <c r="AH1" t="inlineStr">
         <is>
-          <t>top_right_intensity_ratio</t>
+          <t>fwhm_pixel_z_median</t>
         </is>
       </c>
       <c r="AI1" t="inlineStr">
         <is>
-          <t>middle_left_intensity_mean</t>
+          <t>fwhm_pixel_z_std</t>
         </is>
       </c>
       <c r="AJ1" t="inlineStr">
         <is>
-          <t>middle_left_intensity_ratio</t>
+          <t>fwhm_pixel_y_mean</t>
         </is>
       </c>
       <c r="AK1" t="inlineStr">
         <is>
-          <t>middle_center_intensity_mean</t>
+          <t>fwhm_pixel_y_median</t>
         </is>
       </c>
       <c r="AL1" t="inlineStr">
         <is>
-          <t>middle_center_intensity_ratio</t>
+          <t>fwhm_pixel_y_std</t>
         </is>
       </c>
       <c r="AM1" t="inlineStr">
         <is>
-          <t>middle_right_intensity_mean</t>
+          <t>fwhm_pixel_x_mean</t>
         </is>
       </c>
       <c r="AN1" t="inlineStr">
         <is>
-          <t>middle_right_intensity_ratio</t>
+          <t>fwhm_pixel_x_median</t>
         </is>
       </c>
       <c r="AO1" t="inlineStr">
         <is>
-          <t>bottom_left_intensity_mean</t>
+          <t>fwhm_pixel_x_std</t>
         </is>
       </c>
       <c r="AP1" t="inlineStr">
         <is>
-          <t>bottom_left_intensity_ratio</t>
+          <t>fwhm_micron_z_mean</t>
         </is>
       </c>
       <c r="AQ1" t="inlineStr">
         <is>
-          <t>bottom_center_intensity_mean</t>
+          <t>fwhm_micron_z_median</t>
         </is>
       </c>
       <c r="AR1" t="inlineStr">
         <is>
-          <t>bottom_center_intensity_ratio</t>
+          <t>fwhm_micron_z_std</t>
         </is>
       </c>
       <c r="AS1" t="inlineStr">
         <is>
-          <t>bottom_right_intensity_mean</t>
+          <t>fwhm_micron_y_mean</t>
         </is>
       </c>
       <c r="AT1" t="inlineStr">
         <is>
-          <t>bottom_right_intensity_ratio</t>
+          <t>fwhm_micron_y_median</t>
         </is>
       </c>
       <c r="AU1" t="inlineStr">
         <is>
-          <t>table_data</t>
+          <t>fwhm_micron_y_std</t>
         </is>
       </c>
       <c r="AV1" t="inlineStr">
         <is>
-          <t>data_reference</t>
+          <t>fwhm_micron_x_mean</t>
         </is>
       </c>
       <c r="AW1" t="inlineStr">
         <is>
-          <t>linked_references</t>
+          <t>fwhm_micron_x_median</t>
         </is>
       </c>
       <c r="AX1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>fwhm_micron_x_std</t>
         </is>
       </c>
       <c r="AY1" t="inlineStr">
         <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>bead_diameter_micron</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>preparation_protocol</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>preparation_datetime</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>manufacturer</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>sample</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>input_parameters</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>acquisition_datetime</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>input_data</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>output</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>microscope</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>experimenter</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>acquisition_protocol</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>processed</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>data_reference</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>linked_references</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet35.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>psf_beads_images</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet36.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>bit_depth</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>saturation_threshold</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>min_lateral_distance_factor</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sigma_min</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>sigma_max</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>snr_threshold</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>fitting_r2_threshold</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>intensity_robust_z_score_threshold</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:X1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>analyzed_bead_centers</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>considered_bead_centers_lateral_edge</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>considered_bead_centers_self_proximity</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>considered_bead_centers_axial_edge</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>considered_bead_centers_intensity_outlier</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>considered_bead_centers_z_fit_quality</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>considered_bead_centers_y_fit_quality</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>considered_bead_centers_x_fit_quality</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>key_measurements</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>bead_properties</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>bead_profiles_z</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>bead_profiles_y</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>bead_profiles_x</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>average_bead</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>comment</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>processing_application</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>processing_version</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>processing_entity</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>processing_datetime</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>processing_log</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>warnings</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>errors</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>validated</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>validation_datetime</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:BT1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>channel_name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>channel_nr</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>total_bead_count</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>considered_valid_count</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>considered_self_proximity_count</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>considered_lateral_edge_count</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>considered_axial_edge_count</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>considered_intensity_outlier_count</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>considered_bad_fit_z_count</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>considered_bad_fit_y_count</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>considered_bad_fit_x_count</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>intensity_integrated_mean</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>intensity_integrated_median</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>intensity_integrated_std</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>intensity_max_mean</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>intensity_max_median</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>intensity_max_std</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>intensity_min_mean</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>intensity_min_median</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>intensity_min_std</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>intensity_std_mean</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>intensity_std_median</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>intensity_std_std</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>fit_r2_z_mean</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>fit_r2_z_median</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>fit_r2_z_std</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>fit_r2_y_mean</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>fit_r2_y_median</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>fit_r2_y_std</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>fit_r2_x_mean</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>fit_r2_x_median</t>
-        </is>
-      </c>
-      <c r="AF1" t="inlineStr">
-        <is>
-          <t>fit_r2_x_std</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_z_mean</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_z_median</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_z_std</t>
-        </is>
-      </c>
-      <c r="AJ1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_y_mean</t>
-        </is>
-      </c>
-      <c r="AK1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_y_median</t>
-        </is>
-      </c>
-      <c r="AL1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_y_std</t>
-        </is>
-      </c>
-      <c r="AM1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_x_mean</t>
-        </is>
-      </c>
-      <c r="AN1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_x_median</t>
-        </is>
-      </c>
-      <c r="AO1" t="inlineStr">
-        <is>
-          <t>fwhm_pixel_x_std</t>
-        </is>
-      </c>
-      <c r="AP1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_z_mean</t>
-        </is>
-      </c>
-      <c r="AQ1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_z_median</t>
-        </is>
-      </c>
-      <c r="AR1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_z_std</t>
-        </is>
-      </c>
-      <c r="AS1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_y_mean</t>
-        </is>
-      </c>
-      <c r="AT1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_y_median</t>
-        </is>
-      </c>
-      <c r="AU1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_y_std</t>
-        </is>
-      </c>
-      <c r="AV1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_x_mean</t>
-        </is>
-      </c>
-      <c r="AW1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_x_median</t>
-        </is>
-      </c>
-      <c r="AX1" t="inlineStr">
-        <is>
-          <t>fwhm_micron_x_std</t>
-        </is>
-      </c>
-      <c r="AY1" t="inlineStr">
-        <is>
           <t>fwhm_lateral_asymmetry_ratio_mean</t>
         </is>
       </c>
@@ -2830,31 +2805,6 @@
       <c r="BO1" t="inlineStr">
         <is>
           <t>average_bead_intensity_std</t>
-        </is>
-      </c>
-      <c r="BP1" t="inlineStr">
-        <is>
-          <t>table_data</t>
-        </is>
-      </c>
-      <c r="BQ1" t="inlineStr">
-        <is>
-          <t>data_reference</t>
-        </is>
-      </c>
-      <c r="BR1" t="inlineStr">
-        <is>
-          <t>linked_references</t>
-        </is>
-      </c>
-      <c r="BS1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="BT1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -3149,7 +3099,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:V1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3261,31 +3211,6 @@
       <c r="V1" t="inlineStr">
         <is>
           <t>long_term_power_stability</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>table_data</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>data_reference</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>linked_references</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3659,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3756,31 +3681,6 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>saturated_channels</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>table_data</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>data_reference</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>linked_references</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>name</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Removed underscores from MeasuringLocation enum
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3217,7 +3217,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SOURCE_EXIT,FIBER_EXIT,OBJECTIVE_BACKFOCAL,OBJECTIVE_EXIT,OBJECTIVE_FOCAL,OTHER"</formula1>
+      <formula1>"SOURCEEXIT,FIBEREXIT,OBJECTIVEBACKFOCAL,OBJECTIVEEXIT,OBJECTIVEFOCAL,OTHER"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3273,7 +3273,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SOURCE_EXIT,FIBER_EXIT,OBJECTIVE_BACKFOCAL,OBJECTIVE_EXIT,OBJECTIVE_FOCAL,OTHER"</formula1>
+      <formula1>"SOURCEEXIT,FIBEREXIT,OBJECTIVEBACKFOCAL,OBJECTIVEEXIT,OBJECTIVEFOCAL,OTHER"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Revert "Removed underscores from MeasuringLocation enum"
This reverts commit 70f80391
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -3217,7 +3217,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="C2:C1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SOURCEEXIT,FIBEREXIT,OBJECTIVEBACKFOCAL,OBJECTIVEEXIT,OBJECTIVEFOCAL,OTHER"</formula1>
+      <formula1>"SOURCE_EXIT,FIBER_EXIT,OBJECTIVE_BACKFOCAL,OBJECTIVE_EXIT,OBJECTIVE_FOCAL,OTHER"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3273,7 +3273,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="D2:D1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"SOURCEEXIT,FIBEREXIT,OBJECTIVEBACKFOCAL,OBJECTIVEEXIT,OBJECTIVEFOCAL,OTHER"</formula1>
+      <formula1>"SOURCE_EXIT,FIBER_EXIT,OBJECTIVE_BACKFOCAL,OBJECTIVE_EXIT,OBJECTIVE_FOCAL,OTHER"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Added support for differentiating Gaussian and Airy fits in PSF bead analysis schema
</commit_message>
<xml_diff>
--- a/project/excel/microscopemetrics_schema.xlsx
+++ b/project/excel/microscopemetrics_schema.xlsx
@@ -2276,7 +2276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2312,11 +2312,16 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>fitting_r2_threshold</t>
+          <t>fitting_gaussian_r2_threshold</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>fitting_airy_r2_threshold</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>intensity_robust_z_score_threshold</t>
         </is>
       </c>
@@ -2332,7 +2337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:AA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2363,446 +2368,536 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>considered_bead_centers_z_fit_quality</t>
+          <t>considered_bead_centers_z_fit_airy_quality</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>considered_bead_centers_y_fit_quality</t>
+          <t>considered_bead_centers_y_fit_airy_quality</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>considered_bead_centers_x_fit_quality</t>
+          <t>considered_bead_centers_x_fit_airy_quality</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>considered_bead_centers_z_fit_gaussian_quality</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_y_fit_gaussian_quality</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>considered_bead_centers_x_fit_gaussian_quality</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>bead_properties</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>bead_profiles_z</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>bead_profiles_y</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>bead_profiles_x</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>average_bead</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>key_measurements</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>processing_application</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>processing_version</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>processing_entity</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>processing_datetime</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>processing_log</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>warnings</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>errors</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>validated</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>validation_datetime</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:CD1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>channel_name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>channel_nr</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>total_bead_count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>considered_valid_count</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>considered_self_proximity_count</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>considered_lateral_edge_count</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>considered_axial_edge_count</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>considered_intensity_outlier_count</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>considered_bad_fit_airy_z_count</t>
+        </is>
+      </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>bead_profiles_z</t>
+          <t>considered_bad_fit_airy_y_count</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>bead_profiles_y</t>
+          <t>considered_bad_fit_airy_x_count</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>bead_profiles_x</t>
+          <t>considered_bad_fit_gaussian_z_count</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>average_bead</t>
+          <t>considered_bad_fit_gaussian_y_count</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>key_measurements</t>
+          <t>considered_bad_fit_gaussian_x_count</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>comment</t>
+          <t>intensity_integrated_mean</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
         <is>
-          <t>processing_application</t>
+          <t>intensity_integrated_median</t>
         </is>
       </c>
       <c r="Q1" t="inlineStr">
         <is>
-          <t>processing_version</t>
+          <t>intensity_integrated_std</t>
         </is>
       </c>
       <c r="R1" t="inlineStr">
         <is>
-          <t>processing_entity</t>
+          <t>intensity_max_mean</t>
         </is>
       </c>
       <c r="S1" t="inlineStr">
         <is>
-          <t>processing_datetime</t>
+          <t>intensity_max_median</t>
         </is>
       </c>
       <c r="T1" t="inlineStr">
         <is>
-          <t>processing_log</t>
+          <t>intensity_max_std</t>
         </is>
       </c>
       <c r="U1" t="inlineStr">
         <is>
-          <t>warnings</t>
+          <t>intensity_min_mean</t>
         </is>
       </c>
       <c r="V1" t="inlineStr">
         <is>
-          <t>errors</t>
+          <t>intensity_min_median</t>
         </is>
       </c>
       <c r="W1" t="inlineStr">
         <is>
-          <t>validated</t>
+          <t>intensity_min_std</t>
         </is>
       </c>
       <c r="X1" t="inlineStr">
         <is>
-          <t>validation_datetime</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:BO1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>channel_name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>channel_nr</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>total_bead_count</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>considered_valid_count</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>considered_self_proximity_count</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>considered_lateral_edge_count</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>considered_axial_edge_count</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>considered_intensity_outlier_count</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>considered_bad_fit_z_count</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>considered_bad_fit_y_count</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>considered_bad_fit_x_count</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>intensity_integrated_mean</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>intensity_integrated_median</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>intensity_integrated_std</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>intensity_max_mean</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>intensity_max_median</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>intensity_max_std</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>intensity_min_mean</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>intensity_min_median</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>intensity_min_std</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
           <t>intensity_std_mean</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>intensity_std_median</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>intensity_std_std</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>fit_r2_z_mean</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>fit_r2_z_median</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>fit_r2_z_std</t>
-        </is>
-      </c>
       <c r="AA1" t="inlineStr">
         <is>
-          <t>fit_r2_y_mean</t>
+          <t>fit_airy_r2_z_mean</t>
         </is>
       </c>
       <c r="AB1" t="inlineStr">
         <is>
-          <t>fit_r2_y_median</t>
+          <t>fit_airy_r2_z_median</t>
         </is>
       </c>
       <c r="AC1" t="inlineStr">
         <is>
-          <t>fit_r2_y_std</t>
+          <t>fit_airy_r2_z_std</t>
         </is>
       </c>
       <c r="AD1" t="inlineStr">
         <is>
-          <t>fit_r2_x_mean</t>
+          <t>fit_airy_r2_y_mean</t>
         </is>
       </c>
       <c r="AE1" t="inlineStr">
         <is>
-          <t>fit_r2_x_median</t>
+          <t>fit_airy_r2_y_median</t>
         </is>
       </c>
       <c r="AF1" t="inlineStr">
         <is>
-          <t>fit_r2_x_std</t>
+          <t>fit_airy_r2_y_std</t>
         </is>
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>fit_airy_r2_x_mean</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>fit_airy_r2_x_median</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>fit_airy_r2_x_std</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_z_mean</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_z_median</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_z_std</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_y_mean</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_y_median</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_y_std</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_x_mean</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_x_median</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>fit_gaussian_r2_x_std</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
           <t>fwhm_pixel_z_mean</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>fwhm_pixel_z_median</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>fwhm_pixel_z_std</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>fwhm_pixel_y_mean</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>fwhm_pixel_y_median</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>fwhm_pixel_y_std</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>fwhm_pixel_x_mean</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>fwhm_pixel_x_median</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>fwhm_pixel_x_std</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>fwhm_micron_z_mean</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>fwhm_micron_z_median</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>fwhm_micron_z_std</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>fwhm_micron_y_mean</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>fwhm_micron_y_median</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>fwhm_micron_y_std</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>fwhm_micron_x_mean</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>fwhm_micron_x_median</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>fwhm_micron_x_std</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>fwhm_lateral_asymmetry_ratio_mean</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>fwhm_lateral_asymmetry_ratio_median</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>fwhm_lateral_asymmetry_ratio_std</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
-        <is>
-          <t>average_bead_fit_r2_z</t>
-        </is>
-      </c>
-      <c r="BC1" t="inlineStr">
-        <is>
-          <t>average_bead_fit_r2_y</t>
-        </is>
-      </c>
-      <c r="BD1" t="inlineStr">
-        <is>
-          <t>average_bead_fit_r2_x</t>
-        </is>
-      </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
+        <is>
+          <t>average_bead_fit_airy_r2_z</t>
+        </is>
+      </c>
+      <c r="BO1" t="inlineStr">
+        <is>
+          <t>average_bead_fit_airy_r2_y</t>
+        </is>
+      </c>
+      <c r="BP1" t="inlineStr">
+        <is>
+          <t>average_bead_fit_airy_r2_x</t>
+        </is>
+      </c>
+      <c r="BQ1" t="inlineStr">
+        <is>
+          <t>average_bead_fit_gaussian_r2_z</t>
+        </is>
+      </c>
+      <c r="BR1" t="inlineStr">
+        <is>
+          <t>average_bead_fit_gaussian_r2_y</t>
+        </is>
+      </c>
+      <c r="BS1" t="inlineStr">
+        <is>
+          <t>average_bead_fit_gaussian_r2_x</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
         <is>
           <t>average_bead_fwhm_pixel_z</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>average_bead_fwhm_pixel_y</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>average_bead_fwhm_pixel_x</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>average_bead_fwhm_micron_z</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BX1" t="inlineStr">
         <is>
           <t>average_bead_fwhm_micron_y</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BY1" t="inlineStr">
         <is>
           <t>average_bead_fwhm_micron_x</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>average_bead_fwhm_lateral_asymmetry_ratio</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="CA1" t="inlineStr">
         <is>
           <t>average_bead_intensity_integrated</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="CB1" t="inlineStr">
         <is>
           <t>average_bead_intensity_max</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="CC1" t="inlineStr">
         <is>
           <t>average_bead_intensity_min</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="CD1" t="inlineStr">
         <is>
           <t>average_bead_intensity_std</t>
         </is>

</xml_diff>